<commit_message>
54924 Trail Balance Report- Do not treat transaction "transition year" as transaction
Related Work Items: #54924
</commit_message>
<xml_diff>
--- a/Logitude/Logitude.Accounting.BL/CoreBL/Reports/TrailReportBase - Spreadsheet4.xlsx
+++ b/Logitude/Logitude.Accounting.BL/CoreBL/Reports/TrailReportBase - Spreadsheet4.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="9435" yWindow="0" windowWidth="13500" windowHeight="10350"/>
+    <workbookView xWindow="11850" yWindow="0" windowWidth="13500" windowHeight="10350"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>ZERO=BC</t>
   </si>
@@ -208,14 +208,63 @@
     <t>"+1*qYearTransferLedgerTransaction"</t>
   </si>
   <si>
-    <t>"-1*qYearTransferLedgerTransaction"</t>
+    <r>
+      <t>RemoveFrom_</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TransStart</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(qYearTransferLedgerTransaction);</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Add2</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TotalStart</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="177"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(qYearTransferLedgerTransaction);</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -280,6 +329,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -491,12 +548,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -554,7 +612,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -844,9 +903,9 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="7.75" customWidth="1"/>
-    <col min="5" max="5" width="41.75" customWidth="1"/>
+    <col min="3" max="3" width="8.625" customWidth="1"/>
+    <col min="4" max="4" width="32.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="59" customWidth="1"/>
     <col min="8" max="8" width="43" customWidth="1"/>
     <col min="10" max="10" width="42.5" customWidth="1"/>
     <col min="11" max="11" width="12.125" customWidth="1"/>
@@ -885,80 +944,85 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="32" t="s">
+    <row r="3" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="33" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="E6" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="14"/>
+    </row>
+    <row r="7" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E7" s="15"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="17"/>
+    </row>
+    <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E8" s="34" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="E9" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="19"/>
+      <c r="L9" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="M9" s="25"/>
+      <c r="N9" s="26"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="E10" s="20"/>
+      <c r="F10" s="21"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="28"/>
+      <c r="N10" s="29"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="E11" s="20"/>
+      <c r="F11" s="21"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="28"/>
+      <c r="N11" s="29"/>
+    </row>
+    <row r="12" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E12" s="22"/>
+      <c r="F12" s="23"/>
+      <c r="L12" s="30"/>
+      <c r="M12" s="31"/>
+      <c r="N12" s="32"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="E13" s="5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="7"/>
-    </row>
-    <row r="5" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="32" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="E6" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="13"/>
-    </row>
-    <row r="7" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E7" s="14"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="16"/>
-    </row>
-    <row r="8" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="E9" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="18"/>
-      <c r="L9" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="M9" s="24"/>
-      <c r="N9" s="25"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="E10" s="19"/>
-      <c r="F10" s="20"/>
-      <c r="L10" s="26"/>
-      <c r="M10" s="27"/>
-      <c r="N10" s="28"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="E11" s="19"/>
-      <c r="F11" s="20"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="28"/>
-    </row>
-    <row r="12" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E12" s="21"/>
-      <c r="F12" s="22"/>
-      <c r="L12" s="29"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="31"/>
     </row>
     <row r="16" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="E16" s="3" t="s">

</xml_diff>